<commit_message>
Remove k fold cross validation + update test and holdout
</commit_message>
<xml_diff>
--- a/resnet_results.xlsx
+++ b/resnet_results.xlsx
@@ -445,7 +445,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.2088924646377563</v>
+        <v>0.1902019679546356</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>0.1905808299779892</v>
+        <v>0.2009212672710419</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>0.1815811097621918</v>
+        <v>0.1899139583110809</v>
       </c>
     </row>
     <row r="5">
@@ -469,7 +469,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>0.1807550340890884</v>
+        <v>0.1980724185705185</v>
       </c>
     </row>
     <row r="6">
@@ -477,7 +477,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>0.1741297543048859</v>
+        <v>0.1872836798429489</v>
       </c>
     </row>
     <row r="7">
@@ -485,7 +485,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>0.1687377393245697</v>
+        <v>0.1969930976629257</v>
       </c>
     </row>
     <row r="8">
@@ -493,7 +493,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>0.1963492333889008</v>
+        <v>0.1714870631694794</v>
       </c>
     </row>
     <row r="9">
@@ -501,7 +501,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0.1797120422124863</v>
+        <v>0.2038980573415756</v>
       </c>
     </row>
     <row r="10">
@@ -509,7 +509,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>0.1928000301122665</v>
+        <v>0.2066346406936646</v>
       </c>
     </row>
     <row r="11">
@@ -517,7 +517,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>0.2092253714799881</v>
+        <v>0.197903573513031</v>
       </c>
     </row>
     <row r="12">
@@ -528,7 +528,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0.1883 ± 0.0131</t>
+          <t>0.1943 ± 0.0096</t>
         </is>
       </c>
     </row>

</xml_diff>